<commit_message>
Podlahový EPS: 80+50 v celém domě, koupelna 1.20 jen 80 kvůli spádu
</commit_message>
<xml_diff>
--- a/docs/podlaha-eps.xlsx
+++ b/docs/podlaha-eps.xlsx
@@ -576,7 +576,7 @@
         <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G3" t="n">
         <v>8</v>
@@ -585,7 +585,7 @@
         <v>50</v>
       </c>
       <c r="I3" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J3" t="n">
         <v>130</v>
@@ -607,11 +607,11 @@
         <v>2.597</v>
       </c>
       <c r="O3" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G4" t="n">
         <v>8</v>
@@ -647,7 +647,7 @@
         <v>50</v>
       </c>
       <c r="I4" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J4" t="n">
         <v>130</v>
@@ -669,11 +669,11 @@
         <v>7.658</v>
       </c>
       <c r="O4" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G5" t="n">
         <v>8</v>
@@ -709,7 +709,7 @@
         <v>50</v>
       </c>
       <c r="I5" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J5" t="n">
         <v>130</v>
@@ -731,11 +731,11 @@
         <v>0.6919999999999999</v>
       </c>
       <c r="O5" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G6" t="n">
         <v>8</v>
@@ -771,7 +771,7 @@
         <v>50</v>
       </c>
       <c r="I6" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J6" t="n">
         <v>130</v>
@@ -793,11 +793,11 @@
         <v>0.764</v>
       </c>
       <c r="O6" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
         <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G7" t="n">
         <v>8</v>
@@ -833,7 +833,7 @@
         <v>50</v>
       </c>
       <c r="I7" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J7" t="n">
         <v>130</v>
@@ -855,11 +855,11 @@
         <v>3.214</v>
       </c>
       <c r="O7" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
         <v>13</v>
       </c>
       <c r="F8" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="G8" t="n">
         <v>8</v>
@@ -895,14 +895,14 @@
         <v>50</v>
       </c>
       <c r="I8" t="n">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="J8" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>80 + 40</t>
+          <t>80 + 50</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -914,14 +914,14 @@
         <v>2.93</v>
       </c>
       <c r="N8" t="n">
-        <v>0.352</v>
+        <v>0.381</v>
       </c>
       <c r="O8" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Stejný EPS jako dům; potěr 49 mm (o 9 mm tenčí kvůli dlažbě), min. 45 mm nad nopy.</t>
         </is>
       </c>
     </row>
@@ -948,7 +948,7 @@
         <v>13</v>
       </c>
       <c r="F9" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="G9" t="n">
         <v>8</v>
@@ -957,14 +957,14 @@
         <v>50</v>
       </c>
       <c r="I9" t="n">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="J9" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>80 + 40</t>
+          <t>80 + 50</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -976,14 +976,14 @@
         <v>8.91</v>
       </c>
       <c r="N9" t="n">
-        <v>1.069</v>
+        <v>1.158</v>
       </c>
       <c r="O9" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Stejný EPS jako dům; potěr 49 mm (o 9 mm tenčí kvůli dlažbě), min. 45 mm nad nopy.</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
         <v>4</v>
       </c>
       <c r="F10" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G10" t="n">
         <v>8</v>
@@ -1019,7 +1019,7 @@
         <v>50</v>
       </c>
       <c r="I10" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J10" t="n">
         <v>130</v>
@@ -1041,11 +1041,11 @@
         <v>0.6840000000000001</v>
       </c>
       <c r="O10" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
         <v>13</v>
       </c>
       <c r="F11" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="G11" t="n">
         <v>8</v>
@@ -1081,14 +1081,14 @@
         <v>50</v>
       </c>
       <c r="I11" t="n">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="J11" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>80 + 40</t>
+          <t>80 + 50</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1100,14 +1100,14 @@
         <v>6.27</v>
       </c>
       <c r="N11" t="n">
-        <v>0.752</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="O11" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Stejný EPS jako dům; potěr 49 mm (o 9 mm tenčí kvůli dlažbě), min. 45 mm nad nopy.</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
         <v>4</v>
       </c>
       <c r="F12" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G12" t="n">
         <v>8</v>
@@ -1143,7 +1143,7 @@
         <v>50</v>
       </c>
       <c r="I12" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J12" t="n">
         <v>130</v>
@@ -1165,11 +1165,11 @@
         <v>1.228</v>
       </c>
       <c r="O12" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
         <v>4</v>
       </c>
       <c r="F13" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G13" t="n">
         <v>8</v>
@@ -1205,7 +1205,7 @@
         <v>50</v>
       </c>
       <c r="I13" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J13" t="n">
         <v>130</v>
@@ -1227,11 +1227,11 @@
         <v>2.987</v>
       </c>
       <c r="O13" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
         <v>4</v>
       </c>
       <c r="F14" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G14" t="n">
         <v>8</v>
@@ -1267,7 +1267,7 @@
         <v>50</v>
       </c>
       <c r="I14" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J14" t="n">
         <v>130</v>
@@ -1289,11 +1289,11 @@
         <v>1.777</v>
       </c>
       <c r="O14" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1320,7 @@
         <v>4</v>
       </c>
       <c r="F15" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G15" t="n">
         <v>8</v>
@@ -1329,7 +1329,7 @@
         <v>50</v>
       </c>
       <c r="I15" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J15" t="n">
         <v>130</v>
@@ -1351,11 +1351,11 @@
         <v>1.777</v>
       </c>
       <c r="O15" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
         <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G16" t="n">
         <v>8</v>
@@ -1391,7 +1391,7 @@
         <v>50</v>
       </c>
       <c r="I16" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J16" t="n">
         <v>130</v>
@@ -1413,11 +1413,11 @@
         <v>1.777</v>
       </c>
       <c r="O16" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1444,7 @@
         <v>4</v>
       </c>
       <c r="F17" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G17" t="n">
         <v>8</v>
@@ -1453,7 +1453,7 @@
         <v>50</v>
       </c>
       <c r="I17" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J17" t="n">
         <v>130</v>
@@ -1475,11 +1475,11 @@
         <v>2.629</v>
       </c>
       <c r="O17" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
         <v>13</v>
       </c>
       <c r="F21" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="G21" t="n">
         <v>8</v>
@@ -1701,14 +1701,14 @@
         <v>50</v>
       </c>
       <c r="I21" t="n">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="J21" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>80 + 40</t>
+          <t>80 + 50</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1720,14 +1720,14 @@
         <v>2.5</v>
       </c>
       <c r="N21" t="n">
-        <v>0.3</v>
+        <v>0.325</v>
       </c>
       <c r="O21" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Stejný EPS jako dům; potěr 49 mm (o 9 mm tenčí kvůli dlažbě), min. 45 mm nad nopy.</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1754,7 @@
         <v>13</v>
       </c>
       <c r="F22" t="n">
-        <v>60</v>
+        <v>99</v>
       </c>
       <c r="G22" t="n">
         <v>8</v>
@@ -1763,14 +1763,14 @@
         <v>50</v>
       </c>
       <c r="I22" t="n">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="J22" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>80 + 40</t>
+          <t>80</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -1782,14 +1782,14 @@
         <v>4.19</v>
       </c>
       <c r="N22" t="n">
-        <v>0.503</v>
+        <v>0.335</v>
       </c>
       <c r="O22" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Spád 1,5 % k vpusti, rozdíl ~43 mm: potěr 99 mm u dveří → ~56 mm u vpusti (min. 45 nad nopy, rezerva 11). Jedna vrstva 80 (spodní 50 vynechána); přechod ve dveřích = dilatační spára.</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
         <v>13</v>
       </c>
       <c r="F23" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="G23" t="n">
         <v>8</v>
@@ -1825,14 +1825,14 @@
         <v>50</v>
       </c>
       <c r="I23" t="n">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="J23" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>80 + 40</t>
+          <t>80 + 50</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -1844,14 +1844,14 @@
         <v>4.54</v>
       </c>
       <c r="N23" t="n">
-        <v>0.545</v>
+        <v>0.59</v>
       </c>
       <c r="O23" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Stejný EPS jako dům; potěr 49 mm (o 9 mm tenčí kvůli dlažbě), min. 45 mm nad nopy.</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1878,7 @@
         <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
         <v>8</v>
@@ -1887,7 +1887,7 @@
         <v>50</v>
       </c>
       <c r="I24" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J24" t="n">
         <v>130</v>
@@ -1909,11 +1909,11 @@
         <v>0.513</v>
       </c>
       <c r="O24" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1940,7 @@
         <v>4</v>
       </c>
       <c r="F25" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G25" t="n">
         <v>8</v>
@@ -1949,7 +1949,7 @@
         <v>50</v>
       </c>
       <c r="I25" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J25" t="n">
         <v>130</v>
@@ -1971,11 +1971,11 @@
         <v>2.604</v>
       </c>
       <c r="O25" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Potěr 60 mm dle skladby A.</t>
+          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2117,13 +2117,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="D3" t="n">
-        <v>29.34</v>
+        <v>262.86</v>
       </c>
       <c r="E3" t="n">
-        <v>1.174</v>
+        <v>13.143</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2131,16 +2131,16 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>31.1</v>
+        <v>278.63</v>
       </c>
       <c r="H3" t="n">
-        <v>1.244</v>
+        <v>13.932</v>
       </c>
       <c r="I3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J3" t="n">
-        <v>6</v>
+        <v>56</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -2163,13 +2163,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="D4" t="n">
-        <v>237.71</v>
+        <v>267.05</v>
       </c>
       <c r="E4" t="n">
-        <v>11.885</v>
+        <v>21.364</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2177,16 +2177,16 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>251.97</v>
+        <v>283.07</v>
       </c>
       <c r="H4" t="n">
-        <v>12.599</v>
+        <v>22.646</v>
       </c>
       <c r="I4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J4" t="n">
-        <v>51</v>
+        <v>95</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -2205,17 +2205,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EPS 100 S</t>
+          <t>EPS 150 S</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="D5" t="n">
-        <v>267.05</v>
+        <v>76.3</v>
       </c>
       <c r="E5" t="n">
-        <v>21.364</v>
+        <v>3.052</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -2223,27 +2223,23 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>283.07</v>
+        <v>80.88</v>
       </c>
       <c r="H5" t="n">
-        <v>22.646</v>
+        <v>3.235</v>
       </c>
       <c r="I5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J5" t="n">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>Isover EPS 150, TL CZ, desky 1000×500 · https://www.isover.cz/en/documents/technicke-listy/tl-isover-eps-150-cz.pdf</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Balení EPS 100 S převzato z EPS 150 (stejný formát) — ověřit u dodavatele.</t>
-        </is>
-      </c>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2255,13 +2251,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="D6" t="n">
-        <v>76.3</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>3.052</v>
+        <v>3.27</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -2269,13 +2265,13 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>80.88</v>
+        <v>69.31999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>3.235</v>
+        <v>3.466</v>
       </c>
       <c r="I6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J6" t="n">
         <v>14</v>
@@ -2297,13 +2293,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D7" t="n">
-        <v>65.40000000000001</v>
+        <v>10.9</v>
       </c>
       <c r="E7" t="n">
-        <v>3.27</v>
+        <v>1.09</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -2311,17 +2307,17 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>69.31999999999999</v>
+        <v>11.55</v>
       </c>
       <c r="H7" t="n">
-        <v>3.466</v>
+        <v>1.155</v>
       </c>
       <c r="I7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J7" t="n">
         <v>5</v>
       </c>
-      <c r="J7" t="n">
-        <v>14</v>
-      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>Isover EPS 150, TL CZ, desky 1000×500 · https://www.isover.cz/en/documents/technicke-listy/tl-isover-eps-150-cz.pdf</t>
@@ -2330,79 +2326,37 @@
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>EPS 150 S</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>100</v>
-      </c>
-      <c r="D8" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="E8" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>6 %</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>11.55</v>
-      </c>
-      <c r="H8" t="n">
-        <v>1.155</v>
-      </c>
-      <c r="I8" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="J8" t="n">
-        <v>5</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Isover EPS 150, TL CZ, desky 1000×500 · https://www.isover.cz/en/documents/technicke-listy/tl-isover-eps-150-cz.pdf</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr"/>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3">
-        <f>SUM(D3:D8)</f>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="3">
+        <f>SUM(D3:D7)</f>
         <v/>
       </c>
-      <c r="E9" s="3">
-        <f>SUM(E3:E8)</f>
+      <c r="E8" s="3">
+        <f>SUM(E3:E7)</f>
         <v/>
       </c>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3">
-        <f>SUM(G3:G8)</f>
+      <c r="F8" s="3" t="inlineStr"/>
+      <c r="G8" s="3">
+        <f>SUM(G3:G7)</f>
         <v/>
       </c>
-      <c r="H9" s="3">
-        <f>SUM(H3:H8)</f>
+      <c r="H8" s="3">
+        <f>SUM(H3:H7)</f>
         <v/>
       </c>
-      <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="3">
-        <f>SUM(J3:J8)</f>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="3">
+        <f>SUM(J3:J7)</f>
         <v/>
       </c>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2418,7 +2372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2488,72 +2442,120 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nová skladba dům</t>
+          <t>Nová skladba dům (2026-10-14)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>finál 4 (PU) / 13 (dlažba) + potěr 60 + syst. deska 50 + EPS + hydroizolace 8; PE fólie 0,2 zanedbána</t>
+          <t>hydroizolace 8 + EPS 100 S 80+50 (bílý, 2 vrstvy na vazbu) + syst. nopová deska 50 (30 EPS + 20 nopy) + potěr 58 + PU 4 = 250 mm</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nová skladba garáž+chodba 1.17</t>
+          <t>Koupelny 1.06/1.07/1.09/1.19/1.21</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PU 4 + beton 100 + syst. deska 50 + EPS 90 + hydroizolace 8 = 252</t>
+          <t>stejný EPS 80+50 (jedna výška EPS v celém domě); potěr 49 + lepidlo+dlažba 13 = 250 mm; min. potěr nad nopy 45 mm</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Venkovní sklad 1.18</t>
+          <t>Koupelna 1.20 (spád)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>beton 100 (placeholder) + EPS 140 + hydroizolace 8 = 248; předpoklad že 1.18 = venkovní sklad</t>
+          <t>EPS jen 80 (1 vrstva); potěr 99 u dveří / ~56 u vpusti (spád 1,5 %, ~43 mm); dlažba 13. Výškový skok EPS jen ve spodní vrstvě, ve dveřích s dilatační spárou</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Zaokrouhlení</t>
+          <t>Proč 80+50 a ne 1×130</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EPS 128→130 (+2 mm), 119→120 (+1), 88→90 (+2), 142→140 (−2) — vyrovná potěr/beton</t>
+          <t>Petr: vazba spár (2 vrstvy); cena materiálu stejná, práce o pár tisíc dražší</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Rezerva</t>
+          <t>Proč bílý EPS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>6 % prořez</t>
+          <t>Šedý by dal U ~0,18 místo ~0,22 W/m²K, nevyplatí se u podlahy na terénu</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Nová skladba garáž+chodba 1.17</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PU 4 + beton 100 + syst. deska 50 + EPS 90 + hydroizolace 8 = 252</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Venkovní sklad 1.18</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>beton 100 (placeholder) + EPS 140 + hydroizolace 8 = 248; předpoklad že 1.18 = venkovní sklad</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Zaokrouhlení</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Dům: tloušťka potěru dopočtena přesně na 250. Garáž 88→90 (+2), sklad 142→140 (−2) — vyrovná beton</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Rezerva</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>6 % prořez</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>Tepelná izolace</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Projekt měl v domě 170 mm EPS; nově 130/120 + syst. deska (nopová EPS ~20–30 mm). Ověřit vůči PENB.</t>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Projekt měl v domě 170 mm EPS; nově 130 (1.20: 80) + syst. deska (nopová EPS ~20–30 mm). Ověřit vůči PENB.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Podlahový EPS: 60+60 v domě, 1.20 40+40, sprcha 1.07 60+40
</commit_message>
<xml_diff>
--- a/docs/podlaha-eps.xlsx
+++ b/docs/podlaha-eps.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -576,7 +576,7 @@
         <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G3" t="n">
         <v>8</v>
@@ -585,14 +585,14 @@
         <v>50</v>
       </c>
       <c r="I3" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J3" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -604,14 +604,14 @@
         <v>19.98</v>
       </c>
       <c r="N3" t="n">
-        <v>2.597</v>
+        <v>2.398</v>
       </c>
       <c r="O3" t="n">
         <v>250</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G4" t="n">
         <v>8</v>
@@ -647,14 +647,14 @@
         <v>50</v>
       </c>
       <c r="I4" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J4" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -666,14 +666,14 @@
         <v>58.91</v>
       </c>
       <c r="N4" t="n">
-        <v>7.658</v>
+        <v>7.069</v>
       </c>
       <c r="O4" t="n">
         <v>250</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G5" t="n">
         <v>8</v>
@@ -709,14 +709,14 @@
         <v>50</v>
       </c>
       <c r="I5" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J5" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -728,14 +728,14 @@
         <v>5.32</v>
       </c>
       <c r="N5" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.638</v>
       </c>
       <c r="O5" t="n">
         <v>250</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G6" t="n">
         <v>8</v>
@@ -771,14 +771,14 @@
         <v>50</v>
       </c>
       <c r="I6" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J6" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -790,14 +790,14 @@
         <v>5.88</v>
       </c>
       <c r="N6" t="n">
-        <v>0.764</v>
+        <v>0.706</v>
       </c>
       <c r="O6" t="n">
         <v>250</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
         <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G7" t="n">
         <v>8</v>
@@ -833,14 +833,14 @@
         <v>50</v>
       </c>
       <c r="I7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -852,14 +852,14 @@
         <v>24.72</v>
       </c>
       <c r="N7" t="n">
-        <v>3.214</v>
+        <v>2.966</v>
       </c>
       <c r="O7" t="n">
         <v>250</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
         <v>13</v>
       </c>
       <c r="F8" t="n">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="G8" t="n">
         <v>8</v>
@@ -895,14 +895,14 @@
         <v>50</v>
       </c>
       <c r="I8" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J8" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -914,14 +914,14 @@
         <v>2.93</v>
       </c>
       <c r="N8" t="n">
-        <v>0.381</v>
+        <v>0.352</v>
       </c>
       <c r="O8" t="n">
         <v>250</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Stejný EPS jako dům; potěr 49 mm (o 9 mm tenčí kvůli dlažbě), min. 45 mm nad nopy.</t>
+          <t>Stejný EPS jako dům; potěr 59 mm (o 9 mm tenčí kvůli dlažbě).</t>
         </is>
       </c>
     </row>
@@ -933,11 +933,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Koupelna</t>
+          <t>Koupelna (mimo sprchu)</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>8.91</v>
+        <v>6.49</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -948,7 +948,7 @@
         <v>13</v>
       </c>
       <c r="F9" t="n">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="G9" t="n">
         <v>8</v>
@@ -957,14 +957,14 @@
         <v>50</v>
       </c>
       <c r="I9" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J9" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -973,44 +973,44 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>8.91</v>
+        <v>6.49</v>
       </c>
       <c r="N9" t="n">
-        <v>1.158</v>
+        <v>0.779</v>
       </c>
       <c r="O9" t="n">
         <v>250</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Stejný EPS jako dům; potěr 49 mm (o 9 mm tenčí kvůli dlažbě), min. 45 mm nad nopy.</t>
+          <t>Stejný EPS jako dům; potěr 59 mm (o 9 mm tenčí kvůli dlažbě).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>1.07</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Prádelna</t>
+          <t>Koupelna – sprchový kout</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5.26</v>
+        <v>2.42</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PU stěrka 4</t>
+          <t>lepidlo+dlažba 13</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F10" t="n">
-        <v>58</v>
+        <v>79</v>
       </c>
       <c r="G10" t="n">
         <v>8</v>
@@ -1019,14 +1019,14 @@
         <v>50</v>
       </c>
       <c r="I10" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="J10" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 40</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1035,44 +1035,44 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>5.26</v>
+        <v>2.42</v>
       </c>
       <c r="N10" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.242</v>
       </c>
       <c r="O10" t="n">
         <v>250</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Sprchový kout 1.07 (východní, ~1153 × 2100 mm světle; v modelu není samostatná plocha → aproximace 1,153 × 2,1 m). Spád 1,25 % = 26,25 mm: potěr 79 mm na nule → ~53 mm u vpusti.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Koupelna</t>
+          <t>Prádelna</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6.27</v>
+        <v>5.26</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>lepidlo+dlažba 13</t>
+          <t>PU stěrka 4</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="G11" t="n">
         <v>8</v>
@@ -1081,14 +1081,14 @@
         <v>50</v>
       </c>
       <c r="I11" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J11" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1097,44 +1097,44 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>6.27</v>
+        <v>5.26</v>
       </c>
       <c r="N11" t="n">
-        <v>0.8149999999999999</v>
+        <v>0.631</v>
       </c>
       <c r="O11" t="n">
         <v>250</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Stejný EPS jako dům; potěr 49 mm (o 9 mm tenčí kvůli dlažbě), min. 45 mm nad nopy.</t>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Šatna</t>
+          <t>Koupelna</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9.449999999999999</v>
+        <v>6.27</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PU stěrka 4</t>
+          <t>lepidlo+dlažba 13</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F12" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G12" t="n">
         <v>8</v>
@@ -1143,14 +1143,14 @@
         <v>50</v>
       </c>
       <c r="I12" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J12" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1159,33 +1159,33 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>9.449999999999999</v>
+        <v>6.27</v>
       </c>
       <c r="N12" t="n">
-        <v>1.228</v>
+        <v>0.752</v>
       </c>
       <c r="O12" t="n">
         <v>250</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Stejný EPS jako dům; potěr 59 mm (o 9 mm tenčí kvůli dlažbě).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ložnice</t>
+          <t>Šatna</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>22.98</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1196,7 +1196,7 @@
         <v>4</v>
       </c>
       <c r="F13" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G13" t="n">
         <v>8</v>
@@ -1205,14 +1205,14 @@
         <v>50</v>
       </c>
       <c r="I13" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J13" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1221,33 +1221,33 @@
         </is>
       </c>
       <c r="M13" t="n">
-        <v>22.98</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="N13" t="n">
-        <v>2.987</v>
+        <v>1.134</v>
       </c>
       <c r="O13" t="n">
         <v>250</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pokoj</t>
+          <t>Ložnice</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13.67</v>
+        <v>22.98</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         <v>4</v>
       </c>
       <c r="F14" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G14" t="n">
         <v>8</v>
@@ -1267,14 +1267,14 @@
         <v>50</v>
       </c>
       <c r="I14" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J14" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1283,24 +1283,24 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>13.67</v>
+        <v>22.98</v>
       </c>
       <c r="N14" t="n">
-        <v>1.777</v>
+        <v>2.758</v>
       </c>
       <c r="O14" t="n">
         <v>250</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1320,7 +1320,7 @@
         <v>4</v>
       </c>
       <c r="F15" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G15" t="n">
         <v>8</v>
@@ -1329,14 +1329,14 @@
         <v>50</v>
       </c>
       <c r="I15" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J15" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1348,21 +1348,21 @@
         <v>13.67</v>
       </c>
       <c r="N15" t="n">
-        <v>1.777</v>
+        <v>1.64</v>
       </c>
       <c r="O15" t="n">
         <v>250</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1382,7 +1382,7 @@
         <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G16" t="n">
         <v>8</v>
@@ -1391,14 +1391,14 @@
         <v>50</v>
       </c>
       <c r="I16" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J16" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1410,30 +1410,30 @@
         <v>13.67</v>
       </c>
       <c r="N16" t="n">
-        <v>1.777</v>
+        <v>1.64</v>
       </c>
       <c r="O16" t="n">
         <v>250</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Pracovna</t>
+          <t>Pokoj</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>20.22</v>
+        <v>13.67</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1444,7 +1444,7 @@
         <v>4</v>
       </c>
       <c r="F17" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G17" t="n">
         <v>8</v>
@@ -1453,14 +1453,14 @@
         <v>50</v>
       </c>
       <c r="I17" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J17" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1469,33 +1469,33 @@
         </is>
       </c>
       <c r="M17" t="n">
-        <v>20.22</v>
+        <v>13.67</v>
       </c>
       <c r="N17" t="n">
-        <v>2.629</v>
+        <v>1.64</v>
       </c>
       <c r="O17" t="n">
         <v>250</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Garáž</t>
+          <t>Pracovna</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>59.4</v>
+        <v>20.22</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1506,7 +1506,7 @@
         <v>4</v>
       </c>
       <c r="F18" t="n">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="G18" t="n">
         <v>8</v>
@@ -1515,49 +1515,49 @@
         <v>50</v>
       </c>
       <c r="I18" t="n">
-        <v>88</v>
+        <v>120</v>
       </c>
       <c r="J18" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>50 + 40</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>EPS 150 S</t>
+          <t>EPS 100 S</t>
         </is>
       </c>
       <c r="M18" t="n">
-        <v>59.4</v>
+        <v>20.22</v>
       </c>
       <c r="N18" t="n">
-        <v>5.346</v>
+        <v>2.426</v>
       </c>
       <c r="O18" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Nově podlahové topení; beton 100 mm (Petr). Pojezd aut — EPS 150 S min., ověřit se statikem / výrobcem systémové desky (projekt: XPS 80).</t>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Chodba do garáže</t>
+          <t>Garáž</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>6</v>
+        <v>59.4</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1593,10 +1593,10 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>6</v>
+        <v>59.4</v>
       </c>
       <c r="N19" t="n">
-        <v>0.54</v>
+        <v>5.346</v>
       </c>
       <c r="O19" t="n">
         <v>252</v>
@@ -1610,24 +1610,24 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Sklad (venkovní)</t>
+          <t>Chodba do garáže</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>10.9</v>
+        <v>6</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>— (beton)</t>
+          <t>PU stěrka 4</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F20" t="n">
         <v>100</v>
@@ -1636,17 +1636,17 @@
         <v>8</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I20" t="n">
-        <v>142</v>
+        <v>88</v>
       </c>
       <c r="J20" t="n">
-        <v>140</v>
+        <v>90</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>100 + 40</t>
+          <t>50 + 40</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1655,95 +1655,95 @@
         </is>
       </c>
       <c r="M20" t="n">
-        <v>10.9</v>
+        <v>6</v>
       </c>
       <c r="N20" t="n">
-        <v>1.526</v>
+        <v>0.54</v>
       </c>
       <c r="O20" t="n">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Venkovní sklad: jen EPS + beton. Beton 100 mm = PLACEHOLDER (doporučeno 100–120 mm + KARI).</t>
+          <t>Nově podlahové topení; beton 100 mm (Petr). Pojezd aut — EPS 150 S min., ověřit se statikem / výrobcem systémové desky (projekt: XPS 80).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>Sklad (venkovní)</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2.5</v>
+        <v>10.9</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>lepidlo+dlažba 13</t>
+          <t>— (beton)</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>49</v>
+        <v>100</v>
       </c>
       <c r="G21" t="n">
         <v>8</v>
       </c>
       <c r="H21" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="J21" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>100 + 40</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>EPS 100 S</t>
+          <t>EPS 150 S</t>
         </is>
       </c>
       <c r="M21" t="n">
-        <v>2.5</v>
+        <v>10.9</v>
       </c>
       <c r="N21" t="n">
-        <v>0.325</v>
+        <v>1.526</v>
       </c>
       <c r="O21" t="n">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Stejný EPS jako dům; potěr 49 mm (o 9 mm tenčí kvůli dlažbě), min. 45 mm nad nopy.</t>
+          <t>Venkovní sklad: jen EPS + beton. Beton 100 mm = PLACEHOLDER (doporučeno 100–120 mm + KARI).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Koupelna</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4.19</v>
+        <v>2.5</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1754,7 +1754,7 @@
         <v>13</v>
       </c>
       <c r="F22" t="n">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="G22" t="n">
         <v>8</v>
@@ -1763,14 +1763,14 @@
         <v>50</v>
       </c>
       <c r="I22" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="J22" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -1779,24 +1779,24 @@
         </is>
       </c>
       <c r="M22" t="n">
-        <v>4.19</v>
+        <v>2.5</v>
       </c>
       <c r="N22" t="n">
-        <v>0.335</v>
+        <v>0.3</v>
       </c>
       <c r="O22" t="n">
         <v>250</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Spád 1,5 % k vpusti, rozdíl ~43 mm: potěr 99 mm u dveří → ~56 mm u vpusti (min. 45 nad nopy, rezerva 11). Jedna vrstva 80 (spodní 50 vynechána); přechod ve dveřích = dilatační spára.</t>
+          <t>Stejný EPS jako dům; potěr 59 mm (o 9 mm tenčí kvůli dlažbě).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4.54</v>
+        <v>4.19</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1816,7 +1816,7 @@
         <v>13</v>
       </c>
       <c r="F23" t="n">
-        <v>49</v>
+        <v>99</v>
       </c>
       <c r="G23" t="n">
         <v>8</v>
@@ -1825,14 +1825,14 @@
         <v>50</v>
       </c>
       <c r="I23" t="n">
-        <v>130</v>
+        <v>80</v>
       </c>
       <c r="J23" t="n">
-        <v>130</v>
+        <v>80</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>40 + 40</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -1841,44 +1841,44 @@
         </is>
       </c>
       <c r="M23" t="n">
-        <v>4.54</v>
+        <v>4.19</v>
       </c>
       <c r="N23" t="n">
-        <v>0.59</v>
+        <v>0.335</v>
       </c>
       <c r="O23" t="n">
         <v>250</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Stejný EPS jako dům; potěr 49 mm (o 9 mm tenčí kvůli dlažbě), min. 45 mm nad nopy.</t>
+          <t>Diagonální spád k vpusti, rozdíl ~43 mm: potěr 99 mm u dveří → ~56 mm u vpusti (min. 45 nad nopy). Přechod ve dveřích = dilatační spára.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1.22</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Chodba</t>
+          <t>Koupelna</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3.95</v>
+        <v>4.54</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>PU stěrka 4</t>
+          <t>lepidlo+dlažba 13</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G24" t="n">
         <v>8</v>
@@ -1887,14 +1887,14 @@
         <v>50</v>
       </c>
       <c r="I24" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J24" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -1903,33 +1903,33 @@
         </is>
       </c>
       <c r="M24" t="n">
-        <v>3.95</v>
+        <v>4.54</v>
       </c>
       <c r="N24" t="n">
-        <v>0.513</v>
+        <v>0.545</v>
       </c>
       <c r="O24" t="n">
         <v>250</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Stejný EPS jako dům; potěr 59 mm (o 9 mm tenčí kvůli dlažbě).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pokoj+KK</t>
+          <t>Chodba</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>20.03</v>
+        <v>3.95</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1940,7 +1940,7 @@
         <v>4</v>
       </c>
       <c r="F25" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G25" t="n">
         <v>8</v>
@@ -1949,14 +1949,14 @@
         <v>50</v>
       </c>
       <c r="I25" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J25" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>80 + 50</t>
+          <t>60 + 60</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -1965,47 +1965,109 @@
         </is>
       </c>
       <c r="M25" t="n">
-        <v>20.03</v>
+        <v>3.95</v>
       </c>
       <c r="N25" t="n">
-        <v>2.604</v>
+        <v>0.474</v>
       </c>
       <c r="O25" t="n">
         <v>250</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Potěr 58 mm (250 − 8 − 130 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr"/>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1.23</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Pokoj+KK</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>PU stěrka 4</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>4</v>
+      </c>
+      <c r="F26" t="n">
+        <v>68</v>
+      </c>
+      <c r="G26" t="n">
+        <v>8</v>
+      </c>
+      <c r="H26" t="n">
+        <v>50</v>
+      </c>
+      <c r="I26" t="n">
+        <v>120</v>
+      </c>
+      <c r="J26" t="n">
+        <v>120</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>60 + 60</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>EPS 100 S</t>
+        </is>
+      </c>
+      <c r="M26" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="N26" t="n">
+        <v>2.404</v>
+      </c>
+      <c r="O26" t="n">
+        <v>250</v>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Potěr 68 mm (250 − 8 − 120 − 50 − 4). Bílý EPS, 2 vrstvy na vazbu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="C26" s="3">
-        <f>SUM(C3:C25)</f>
+      <c r="C27" s="3">
+        <f>SUM(C3:C26)</f>
         <v/>
       </c>
-      <c r="D26" s="3" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="3" t="inlineStr"/>
-      <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="3" t="inlineStr"/>
-      <c r="I26" s="3" t="inlineStr"/>
-      <c r="J26" s="3" t="inlineStr"/>
-      <c r="K26" s="3" t="inlineStr"/>
-      <c r="L26" s="3" t="inlineStr"/>
-      <c r="M26" s="3" t="inlineStr"/>
-      <c r="N26" s="3">
-        <f>SUM(N3:N25)</f>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr"/>
+      <c r="J27" s="3" t="inlineStr"/>
+      <c r="K27" s="3" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr"/>
+      <c r="M27" s="3" t="inlineStr"/>
+      <c r="N27" s="3">
+        <f>SUM(N3:N26)</f>
         <v/>
       </c>
-      <c r="O26" s="3" t="n"/>
-      <c r="P26" s="3" t="n"/>
+      <c r="O27" s="3" t="n"/>
+      <c r="P27" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2117,13 +2179,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D3" t="n">
-        <v>262.86</v>
+        <v>10.8</v>
       </c>
       <c r="E3" t="n">
-        <v>13.143</v>
+        <v>0.432</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2131,16 +2193,16 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>278.63</v>
+        <v>11.45</v>
       </c>
       <c r="H3" t="n">
-        <v>13.932</v>
+        <v>0.458</v>
       </c>
       <c r="I3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J3" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -2163,13 +2225,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="D4" t="n">
-        <v>267.05</v>
+        <v>523.3</v>
       </c>
       <c r="E4" t="n">
-        <v>21.364</v>
+        <v>31.398</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2177,16 +2239,16 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>283.07</v>
+        <v>554.7</v>
       </c>
       <c r="H4" t="n">
-        <v>22.646</v>
+        <v>33.282</v>
       </c>
       <c r="I4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J4" t="n">
-        <v>95</v>
+        <v>139</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -2442,12 +2504,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nová skladba dům (2026-10-14)</t>
+          <t>Nová skladba dům (2026-10-14 odp.)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>hydroizolace 8 + EPS 100 S 80+50 (bílý, 2 vrstvy na vazbu) + syst. nopová deska 50 (30 EPS + 20 nopy) + potěr 58 + PU 4 = 250 mm</t>
+          <t>hydroizolace 8 + EPS 100 S 60+60 (bílý, na vazbu) + syst. nopová deska 50 (30 EPS + 20 nopy) + potěr 68 + PU 4 = 250 mm</t>
         </is>
       </c>
     </row>
@@ -2459,67 +2521,67 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>stejný EPS 80+50 (jedna výška EPS v celém domě); potěr 49 + lepidlo+dlažba 13 = 250 mm; min. potěr nad nopy 45 mm</t>
+          <t>EPS 60+60 + deska 50 + potěr 59 + lepidlo+dlažba 13 = 250 mm</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Koupelna 1.20 (spád)</t>
+          <t>Proč 68 / 59</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EPS jen 80 (1 vrstva); potěr 99 u dveří / ~56 u vpusti (spád 1,5 %, ~43 mm); dlažba 13. Výškový skok EPS jen ve spodní vrstvě, ve dveřích s dilatační spárou</t>
+          <t>Dopočet na 250: 250 − 8 − 120 − 50 − finál (4 PU / 13 dlažba). Oba potěry nad min. 45 mm nad nopy</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Proč 80+50 a ne 1×130</t>
+          <t>Proč 60+60</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Petr: vazba spár (2 vrstvy); cena materiálu stejná, práce o pár tisíc dražší</t>
+          <t>Jedna tloušťka desky k nákupu (méně prořezu a záměn), dvě vrstvy kvůli vazbě spár; bílý EPS (šedý se u podlahy na terénu nevyplatí)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Proč bílý EPS</t>
+          <t>Koupelna 1.20 (spád)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Šedý by dal U ~0,18 místo ~0,22 W/m²K, nevyplatí se u podlahy na terénu</t>
+          <t>EPS 40+40; potěr 99 u dveří / ~56 u vpusti (diagonální spád, ~43 mm); skok EPS ve dveřích s dilatační spárou</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Nová skladba garáž+chodba 1.17</t>
+          <t>Sprcha 1.07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PU 4 + beton 100 + syst. deska 50 + EPS 90 + hydroizolace 8 = 252</t>
+          <t>Jen východní sprchový kout ~1153 × 2100 mm (aproximace 1,153 × 2,1 = 2,42 m², v modelu není dílčí plocha): EPS 60+40, potěr 79 na nule / ~53 u vpusti (1,25 % = 26,25 mm); zbytek 1.07 60+60</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Venkovní sklad 1.18</t>
+          <t>Garáž, chodba 1.17, sklad 1.18</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>beton 100 (placeholder) + EPS 140 + hydroizolace 8 = 248; předpoklad že 1.18 = venkovní sklad</t>
+          <t>Beze změny; celkové skladby garáž+1.17 = 252 mm, sklad 1.18 = 248 mm (zaokrouhlení EPS na prodejné desky)</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2593,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dům: tloušťka potěru dopočtena přesně na 250. Garáž 88→90 (+2), sklad 142→140 (−2) — vyrovná beton</t>
+          <t>Dům: potěr dopočten přesně na 250. Garáž 88→90 (+2), sklad 142→140 (−2) — vyrovná beton</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2617,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Projekt měl v domě 170 mm EPS; nově 130 (1.20: 80) + syst. deska (nopová EPS ~20–30 mm). Ověřit vůči PENB.</t>
+          <t>Projekt měl v domě 170 mm EPS; nově 120 (1.20: 80, sprcha 1.07: 100) + syst. deska (nopová EPS ~20–30 mm). Ověřit vůči PENB.</t>
         </is>
       </c>
     </row>

</xml_diff>